<commit_message>
Replace 김현진 W31 with sales/package + Sangji grant directive
Move-in/out package productization, CRM build, consultation/quote/
contract process, partner sales, pipeline tracking, end-to-end test,
and Sangji Univ. 1M-won ad-subsidy application (top priority). Expand
to 8 tasks with report sheet, sums, validations, approval block realigned.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_김현진_2026-W31.xlsx
+++ b/out/BRING_주간_김현진_2026-W31.xlsx
@@ -1544,7 +1544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K47"/>
+  <dimension ref="B1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" customWidth="1" style="49" min="2" max="2"/>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E5" s="110" t="inlineStr">
         <is>
-          <t>운영관리팀장</t>
+          <t>운영관리팀장 / 입·퇴실 패키지 영업 관리</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
@@ -1693,9 +1693,9 @@
       </c>
       <c r="C8" s="70" t="inlineStr">
         <is>
-          <t>이번 주부터 김현진 담당자는 '운영관리팀장' 역할을 조금씩 맡습니다. 대표는 회사의 큰 방향과 이번 주 핵심 목표를 제시하고, 현진 팀장은 운영관리 영역에서 세부 실행방법과 우선순위를 스스로 판단해 실행하고, 진행하며 발견한 문제를 개선하고, 다음에 필요한 일을 먼저 제안하는 구조로 전환합니다.
-아직 회사 운영 전체를 독립적으로 책임지는 단계(COO)는 아닙니다. '방향은 대표가 줄 테니, 운영관리는 팀장으로 조금씩 맡아 세부 방법과 다음 행동을 스스로 생각해보자. 부족한 부분은 대표와 함께 맞춘다'가 이번 단계의 메시지입니다.
-운영관리팀장의 핵심 책임은 '브링에서 발생하는 운영업무가 누락되지 않고 접수부터 완료까지 원활히 연결되도록 관리하는 것'입니다. 모든 일을 직접 하는 것이 아니라, 무엇이 발생했고·무엇을 해야 하고·언제까지·어디까지 됐고·다음 행동이 무엇인지를 관리하는 역할입니다.</t>
+          <t>김현진 팀장은 입·퇴실 패키지 상품화부터 고객 상담·견적·계약까지 영업 전 과정을 관리합니다. 추가로 상지대학교 광고비 100만 원 지원금 신청서 작성 및 제출 준비를 담당합니다.
+지금은 입·퇴실 패키지가 '판매 가능한 상품'으로 정리되어 있지 않고 고객 문의가 체계적으로 관리되지 않습니다. 이번 주에는 패키지를 바로 설명·판매할 수 있는 형태로 완성하고, CRM으로 문의부터 상담·견적·계약까지 관리하는 기반을 만들며, 마감이 있는 상지대 광고비 지원 신청을 준비합니다.
+한 문장으로: 입·퇴실 패키지를 판매 가능한 상품으로 완성하고, CRM으로 문의~계약을 관리하며, 잠재고객·제휴처 영업과 상지대 광고비 지원 신청을 담당합니다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>대표가 제시한 이번 주 핵심 목표를 달성하면서, 운영관리 영역에서 세부 방법·우선순위를 스스로 판단해 실행하고, 발견한 문제를 개선하며 다음 주 할 일을 먼저 제안합니다.</t>
+          <t>입·퇴실 패키지를 바로 판매·설명할 수 있는 상품으로 완성하고, CRM으로 문의~상담~견적~계약을 관리하며, 상지대 광고비 100만 원 지원 신청서를 준비하는 것입니다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C10" s="73" t="inlineStr">
         <is>
-          <t>운영업무 중 빠지거나 멈춘 일이 방치되면 고객·협력업체 대응이 늦어지고 대표 개인에게 계속 의존하게 됩니다. 또한 실행하며 문제를 발견·개선하고 다음 일을 스스로 제안하지 않으면, 매번 대표의 지시를 기다리는 구조가 반복됩니다.</t>
+          <t>패키지가 상품으로 정리되지 않으면 문의가 와도 즉시 판매·견적이 어렵고, CRM 없이 관리하면 상담·견적·재연락이 누락됩니다. 또한 상지대 광고비 지원은 마감이 있어 준비가 늦으면 100만 원 지원 기회를 놓칩니다.</t>
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="C14" s="111" t="inlineStr">
         <is>
-          <t>① 대표 지정 핵심과제 — 목표·이유·완료조건 중심으로 수행 (세부 방법은 팀장 판단)</t>
+          <t>1. 입·퇴실 패키지 상품화 (상품정의서·고객용 소개서·상담문구·가격/옵션표)</t>
         </is>
       </c>
       <c r="D14" s="41" t="n"/>
@@ -1808,7 +1808,7 @@
       <c r="B15" s="112" t="n"/>
       <c r="C15" s="111" t="inlineStr">
         <is>
-          <t>② 주간 운영관리 — 진행 중 운영업무에 빠지거나 멈춘 일이 없는지 점검</t>
+          <t>2. CRM 구축·관리 (진행 14단계·필수 입력정보·관리 기준 적용)</t>
         </is>
       </c>
       <c r="D15" s="41" t="n"/>
@@ -1824,7 +1824,7 @@
       <c r="B16" s="112" t="n"/>
       <c r="C16" s="111" t="inlineStr">
         <is>
-          <t>③ 운영 문제 발견·개선 — 반복·불편 문제를 스스로 찾아 개선</t>
+          <t>3. 고객 상담 (확인사항·상담 후 처리·상담 문구 세트)</t>
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
@@ -1840,7 +1840,7 @@
       <c r="B17" s="112" t="n"/>
       <c r="C17" s="111" t="inlineStr">
         <is>
-          <t>④ 미래 운영 준비 — 규모 확대·사전 준비·대표 업무 이관 관점 검토</t>
+          <t>4. 견적 및 계약 진행 (견적 전 확인·발송 후 관리·계약 확정 절차)</t>
         </is>
       </c>
       <c r="D17" s="41" t="n"/>
@@ -1856,7 +1856,7 @@
       <c r="B18" s="112" t="n"/>
       <c r="C18" s="111" t="inlineStr">
         <is>
-          <t>⑤ 다음 업무 선제 제안 — 다음 주 할 일을 먼저 제안</t>
+          <t>5. 잠재고객·제휴처 영업 (대상·기록항목·제안내용)</t>
         </is>
       </c>
       <c r="D18" s="41" t="n"/>
@@ -1872,7 +1872,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>세부 실행방법·조사방법·접촉방법은 담당자(팀장)가 판단 (대표는 HOW까지 지정하지 않음)</t>
+          <t>6. 문의~계약 전체 진행상황 관리 (매일 점검·지연고객 관리)</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1886,7 +1886,11 @@
     </row>
     <row r="20" ht="39.75" customHeight="1" s="49">
       <c r="B20" s="112" t="n"/>
-      <c r="C20" s="111" t="n"/>
+      <c r="C20" s="111" t="inlineStr">
+        <is>
+          <t>7. 입·퇴실 패키지 전체 과정 테스트 (가상고객 1건 end-to-end)</t>
+        </is>
+      </c>
       <c r="D20" s="41" t="n"/>
       <c r="E20" s="41" t="n"/>
       <c r="F20" s="41" t="n"/>
@@ -1898,7 +1902,11 @@
     </row>
     <row r="21" ht="33.75" customHeight="1" s="49">
       <c r="B21" s="112" t="n"/>
-      <c r="C21" s="113" t="n"/>
+      <c r="C21" s="113" t="inlineStr">
+        <is>
+          <t>8. 상지대학교 광고비 100만 원 지원금 신청 (마감 확인·초안·첨부·검수)</t>
+        </is>
+      </c>
       <c r="D21" s="41" t="n"/>
       <c r="E21" s="41" t="n"/>
       <c r="F21" s="41" t="n"/>
@@ -1916,11 +1924,12 @@
       </c>
       <c r="C22" s="105" t="inlineStr">
         <is>
-          <t>· 고객 직접 연락·상담 (대표가 담당)
-· 타 팀원의 업무·역할 관리 (이번 범위 아님)
-· 이미 만든 CRM의 이유 없는 재구축 / FM 전체구조 반복 설계 / 매주 새 시스템 개발
-· 실제 필요성이 확인되지 않은 자동화 추가 / 학습 자체가 목적인 강의
-· 회사 전체 전략의 단독 판단 / 가용시간을 초과하는 과도한 업무</t>
+          <t>대표 확인/승인 후에만 진행:
+· 가격 변경·할인 (견적 가격 변경은 대표 승인 후)
+· 제휴 조건·소개 수수료 확정
+· 외부 기관(상지대 등) 최종 제출
+· 개인정보 포함 자료의 공개 링크 사용 (금지)
+· 계약 실패 고객 정보 삭제 (삭제 금지 — 실패 이유 기록)</t>
         </is>
       </c>
       <c r="D22" s="41" t="n"/>
@@ -1944,11 +1953,11 @@
       </c>
       <c r="C23" s="105" t="inlineStr">
         <is>
-          <t>· 대표는 방향과 이번 주 핵심 목표를 제시하고, 세부 실행방법·우선순위는 팀장이 판단합니다
-· 자율 영역이라도 '완료조건'은 무엇이 되면 끝인지 산출물·상태로 명확히 남깁니다
-· 이미 만든 시스템(CRM 등)은 '실사용 → 문제발견 → 필요할 때 개선' 방식으로 발전시킵니다
-· 김현진은 학생 신분으로 가용시간이 변동될 수 있으므로, 가용시간 내에서 중요도가 높은 업무부터 수행하고 초과분은 다음 주 후보로 미룹니다
-· 세부 마감은 별도로 두지 않고, 금요일 주간보고로 결과를 정리합니다</t>
+          <t>· 모든 고객에게 반드시 3가지: ① 현재 진행상태 ② 담당자 ③ 다음 행동·예정일
+· 신규 문의는 당일 CRM 등록, 상담 후 주요 내용 즉시 기록, 계약 실패도 삭제하지 말고 이유 기록
+· 매일 확인: 신규/미답변 문의·정보 대기 고객·작성/미발송 견적·재연락 예정·계약 대기·일정 조율·대표 결정 필요
+· 학생 신분으로 가용시간이 변동될 수 있으므로 중요도 높은 업무(상지대 지원 마감·패키지·CRM)부터 하고, 초과분은 다음 주로 이월
+· 세부 마감은 별도로 두지 않고 금요일 주간보고로 정리 (단, 상지대 지원은 공고 마감을 우선)</t>
         </is>
       </c>
       <c r="D23" s="41" t="n"/>
@@ -1972,7 +1981,7 @@
       </c>
       <c r="C24" s="102" t="inlineStr">
         <is>
-          <t>진행 중 범위를 벗어나거나 대표 판단이 필요한 사항이 생기면, 상황을 간단히 정리해 대표와 상의 후 진행합니다.</t>
+          <t>진행 중 대표 판단·승인이 필요하거나 범위를 벗어나는 사항이 생기면, 상황을 정리해 대표에게 보고 후 진행합니다.</t>
         </is>
       </c>
       <c r="D24" s="41" t="n"/>
@@ -2066,25 +2075,24 @@
       </c>
       <c r="C28" s="47" t="inlineStr">
         <is>
-          <t>[핵심과제] 실제 운영에 바로 쓸 협력업체 공급망 확보 (누수·입주청소)</t>
+          <t>입·퇴실 패키지 상품화</t>
         </is>
       </c>
       <c r="D28" s="47" t="inlineStr">
         <is>
-          <t>지난주에 마무리하지 못한 누수·입주청소 협력업체 확보를 이번 주 핵심과제로 완결합니다. 목표는 '실제 운영에 바로 연결해 쓸 수 있는 공급망'이며, 몇 곳을 어떻게 조사·접촉할지 등 구체적 방법은 팀장이 판단합니다.</t>
+          <t>입·퇴실 패키지를 고객에게 바로 설명·판매할 수 있는 형태로 정리합니다.</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>① 누수: 고객 요청 건에 대해 같은 현장조건으로 실제 비교 가능한 견적을 확보하고, 바로 연결 가능한 주력업체 1곳·예비 1곳을 확정합니다(선정 이유·주의사항 포함).
-② 입주청소: 원주에서 지속 협업 가능한 주력 2곳·예비 2곳을 확정하고 실제 단가·조건(단가·추가비용·세금계산서·대응·재작업/AS)을 확인합니다.
-③ 각 선정은 가격·품질·대응속도·신뢰도를 종합해 판단하고, 위험요소와 '바로 연락 가능한 상태'를 함께 정리합니다.
-④ 결과는 표로 정리해 대표가 바로 활용할 수 있게 제공합니다.</t>
+          <t>① 대상 고객(건물주·임대인·관리자·공인중개사·입주/퇴실 예정 고객)과 적용 대상(상가·사무실·원룸/오피스텔·소형건물)을 정의합니다.
+② 기본 서비스 범위·추가 옵션·제외 항목, 입실/퇴실 패키지 차이, 진행 순서·소요시간·가능 지역·고객 준비사항·완료 결과물·문제 처리 기준을 정리합니다.
+③ 산출물을 만듭니다: 내부용 상품정의서 / 고객용 1페이지 소개서 / 상담용 설명문 / 진행순서 안내 / FAQ / 기본가격·추가옵션표 / 고객 필수정보 목록.</t>
         </is>
       </c>
       <c r="F28" s="47" t="inlineStr">
         <is>
-          <t>01_김현진_협력업체_공급망_W31_v1.xlsx</t>
+          <t>01_김현진_입퇴실패키지_상품화_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -2099,14 +2107,14 @@
       </c>
       <c r="I28" s="47" t="inlineStr">
         <is>
-          <t>최우선</t>
+          <t>높음</t>
         </is>
       </c>
       <c r="J28" s="114" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.5</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="29" ht="123" customHeight="1" s="49">
@@ -2115,24 +2123,24 @@
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>[주간 운영관리] 운영업무 점검 — 빠지거나 멈춘 일 확인</t>
+          <t>CRM 구축 및 관리</t>
         </is>
       </c>
       <c r="D29" s="47" t="inlineStr">
         <is>
-          <t>이번 주 진행 중인 운영업무를 훑어 누락·정체된 일이 없는지 확인합니다. 지금 있는 것만 가볍게 점검하면 되며, 없는 데이터를 새로 만들 필요는 없습니다.</t>
+          <t>정리한 업무 흐름을 CRM에 실제로 적용해 고객을 단계별로 관리합니다.</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>① 관리건물·민원·입퇴실·수리/유지보수·협력업체·프로젝트·미완료 업무 등 현재 진행 중인 운영업무를 한 곳에 정리합니다.
-② 각 건에 대해 최소한 담당 / 기한 / 현재상태 / 다음 행동을 파악합니다.
-③ 지연되었거나 멈춘 일, 확인이 필요한 일을 표시합니다.</t>
+          <t>① CRM 진행 14단계(잠재→신규문의→상담→현장정보→견적준비→견적발송→검토→계약확정→일정조율→서비스진행→완료확인→결제완료→리뷰요청→사후관리)를 반영합니다.
+② 고객별 필수 입력정보(고객명·연락처·유형·건물/주소/용도·면적·층수·입퇴실 예정일·필요 서비스·채널·상담내용·견적/계약금액·진행상태·담당자·다음연락일·서류/사진 링크·특이사항·계약여부·실패이유)를 정의합니다.
+③ 관리 기준을 적용합니다: 신규 당일 등록·담당자 지정·다음 연락일 입력·상담 즉시 기록·계약 실패도 이유 기록·개인정보는 공개 링크 금지.</t>
         </is>
       </c>
       <c r="F29" s="47" t="inlineStr">
         <is>
-          <t>02_김현진_주간운영관리_점검_W31_v1.xlsx</t>
+          <t>02_김현진_CRM_구축관리_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2151,10 +2159,10 @@
         </is>
       </c>
       <c r="J29" s="114" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="30" ht="84" customHeight="1" s="49">
@@ -2163,24 +2171,24 @@
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>[문제 발견·개선] 운영 문제 1개 이상 스스로 발굴·개선</t>
+          <t>고객 상담 프로세스·문구 정비</t>
         </is>
       </c>
       <c r="D30" s="47" t="inlineStr">
         <is>
-          <t>업무를 진행하며 지금 운영에서 가장 불편하거나 반복적으로 발생하는 문제를 스스로 찾아 개선합니다. 거대한 시스템을 새로 만들 필요는 없고 작은 문제부터 개선합니다.</t>
+          <t>문의가 오면 고객 상황을 정확히 파악하고 필요한 정보를 CRM에 기록할 수 있도록 상담 체계를 만듭니다.</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>① 반복·불편 문제를 최소 1개 직접 찾습니다.
-② 문제 → 원인 → 개선안 순으로 정리합니다.
-③ 가능하면 이번 주에 적용해 보고 결과까지 확인합니다(적용이 어려우면 개선안·적용계획까지).</t>
+          <t>① 상담 시 확인할 내용(입실/퇴실·위치·유형·면적·희망일·현장상태·청소범위·폐기물·추가서비스·주차/출입·엘리베이터·사진 제공·예산/완료기준)을 체크리스트로 정리합니다.
+② 상담 후 처리(상담 기록·요청사항 요약·추가 사진/서류 요청·현장방문 판단·견적 담당/일정 지정·다음 과정 안내·다음 연락일 등록)를 정합니다.
+③ 상담 문구 세트(첫 문의 답변·부재 시 문자·사진 요청·추가정보 요청·현장방문 제안·견적 발송/확인·보류 재연락·계약 확정·일정 안내·완료 후 리뷰 요청)를 작성합니다.</t>
         </is>
       </c>
       <c r="F30" s="47" t="inlineStr">
         <is>
-          <t>03_김현진_운영문제_개선_W31_v1.pdf</t>
+          <t>03_김현진_상담_프로세스_문구_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2195,7 +2203,7 @@
       </c>
       <c r="I30" s="47" t="inlineStr">
         <is>
-          <t>보통</t>
+          <t>높음</t>
         </is>
       </c>
       <c r="J30" s="114" t="n">
@@ -2211,23 +2219,24 @@
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
-          <t>[미래 준비] 운영 확장 대비 관점 검토</t>
+          <t>견적 및 계약 진행 정비</t>
         </is>
       </c>
       <c r="D31" s="47" t="inlineStr">
         <is>
-          <t>다음 질문 중 하나 이상을 생각해, 실제 준비할 가치가 있는 것을 제안합니다.</t>
+          <t>견적 작성·발송·계약 확정 절차를 정비합니다.</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>① '관리건물이 늘어나면 지금 방식에서 무엇이 가장 먼저 문제가 될까?' / '지금 미리 준비해두면 좋은 것은?' / '대표가 지금 직접 하지만 향후 운영관리로 가져와야 할 업무는?' 중 하나 이상을 검토합니다.
-② 검토 내용 중 준비할 가치가 있는 것을 개선안 또는 다음 업무로 제안합니다.</t>
+          <t>① 견적 전 확인사항(서비스 범위·면적·오염상태·난이도·인원·작업시간·외주/협력비·소모품·이동·폐기물·옵션·예상 원가/마진)을 정리합니다.
+② 견적 발송 후 관리(CRM 견적금액·견적서 링크·발송일·유효기간·고객 확인·익일 확인·3일 후 재연락·할인요청 기록·가격변경은 대표 승인·실패 이유 기록)를 정합니다.
+③ 계약 확정 후 절차(계약금액 확정·범위 재확인·일정·결제방식·고객 준비사항 안내·문서 CRM 연결·담당자 전달·변경/취소 조건 안내)를 정리합니다.</t>
         </is>
       </c>
       <c r="F31" s="47" t="inlineStr">
         <is>
-          <t>04_김현진_미래운영_준비검토_W31_v1.pdf</t>
+          <t>04_김현진_견적계약_진행정비_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G31" s="108" t="inlineStr">
@@ -2246,7 +2255,7 @@
         </is>
       </c>
       <c r="J31" s="114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K31" s="19" t="n">
         <v>0.1</v>
@@ -2258,24 +2267,24 @@
       </c>
       <c r="C32" s="47" t="inlineStr">
         <is>
-          <t>[선제 제안] 다음 주 할 일 2~3개 제안</t>
+          <t>잠재고객·제휴처 영업</t>
         </is>
       </c>
       <c r="D32" s="47" t="inlineStr">
         <is>
-          <t>이번 주를 '업무 완료'로 끝내지 말고, '이걸 끝냈으니 다음으로 무엇을 해야 하는가'를 생각해 다음 주 업무를 먼저 제안합니다.</t>
+          <t>우선 영업 대상과 제휴처를 등록하고 영업을 시작합니다. 제휴 조건·소개 수수료는 대표 보고 후 결정합니다.</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>① 다음 주에 필요하다고 판단하는 업무를 최소 2~3개 제안합니다.
-② 각 제안에 우선순위와 이유, 예상 완료결과를 함께 적습니다.
-③ 금요일 주간보고에 포함합니다.</t>
+          <t>① 우선 대상(건물주·임대인·관리업체·공인중개사·오피스텔 관리자·이사/청소/인테리어/폐기물 업체·이전 예정 사업자)을 등록합니다.
+② 대상별 기록(업체/고객명·지역·담당자·연락처·업종·예상 서비스·제휴 가능성·첫 연락일·상담내용·반응·자료 발송·다음 연락일·제휴 조건·실적)을 관리합니다.
+③ 제휴 제안 내용(고객 연결·공동 안내·상호 소개·서비스별 협력·소개비/제휴 방식·장기 협력)을 준비하되, 조건·수수료는 대표 보고 후 확정합니다.</t>
         </is>
       </c>
       <c r="F32" s="47" t="inlineStr">
         <is>
-          <t>05_김현진_다음주_제안_W31_v1.pdf</t>
+          <t>05_김현진_잠재고객_제휴영업_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G32" s="108" t="inlineStr">
@@ -2294,129 +2303,224 @@
         </is>
       </c>
       <c r="J32" s="114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" s="19" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1" s="49">
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>문의~계약 전체 진행상황 관리</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>문의 응대에 그치지 않고 각 고객이 현재 어디까지 진행됐는지 계속 관리합니다.</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>① 매일 점검(신규/미답변 문의·정보 대기·작성/미발송 견적·재연락 예정·계약 대기·일정 조율·대표 결정 필요)을 수행합니다.
+② 모든 고객에 3요소(진행상태·담당자·다음 행동/예정일)를 유지합니다.
+③ 지연 고객(무응답·자료 미제공·견적 후 무응답·계약 보류·일정 미확정)에 재연락 날짜를 정하고 결과를 CRM에 기록합니다.</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>06_김현진_진행상황_관리_W31_v1.xlsx</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H33" s="107" t="inlineStr">
+        <is>
+          <t>07-31(금) 17:00</t>
+        </is>
+      </c>
+      <c r="I33" s="47" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="J33" s="114" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="19" t="n">
         <v>0.08</v>
       </c>
     </row>
-    <row r="33" ht="69" customHeight="1" s="49">
-      <c r="B33" s="45" t="inlineStr">
+    <row r="34" ht="90" customHeight="1" s="49">
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>입·퇴실 패키지 전체 과정 테스트</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="inlineStr">
+        <is>
+          <t>실제 또는 가상 고객 1건을 CRM에 등록해 전체 과정을 시험하고 개선점을 반영합니다.</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>① 신규 문의→기본정보→상담→현장정보/사진→견적 작성/발송→계약 확정→일정→서비스 진행→완료 자료→결제 완료→리뷰 요청→사후관리까지 1건을 끝까지 진행합니다.
+② 테스트 중 확인(빠진 정보·중복 항목·불명확한 단계·없는 서류/안내문·담당자 미지정·설명 어려운 내용·대표 승인 필요 지점)을 정리합니다.
+③ 결과를 CRM·업무 흐름에 반영합니다.</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>07_김현진_패키지_전과정_테스트_W31_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H34" s="107" t="inlineStr">
+        <is>
+          <t>07-31(금) 17:00</t>
+        </is>
+      </c>
+      <c r="I34" s="47" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="J34" s="114" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1" s="49">
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>상지대학교 광고비 100만 원 지원금 신청  (마감 우선)</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>전달받은 신청서·공고문을 확인해 광고비 100만 원 지원 신청서를 작성하고 제출을 준비합니다. 마감이 있으므로 우선 처리합니다.</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>① 먼저 확인: 지원사업명·지원금액·대상·신청 마감일·제출방법·가능 광고채널·자부담·집행기간·선결제/부가세·정산방식.
+② 신청서 초안 작성(회사/대표/사업자 정보·신청 목적·서비스 및 입퇴실 패키지 소개·광고 필요성·목표 고객·채널·100만 원 사용계획·기간·기대효과·예상 문의/계약 수·성과관리 방법).
+③ 첨부서류 확보(사업자등록증·통장사본·회사소개서·광고 견적서·집행계획서·개인정보 동의서·신청서 등)와 제출 전 검수(누락·회사/대표/사업자번호·예산 합계·기간·서명·파일명·형식·마감).
+④ 최종본을 대표에게 먼저 확인받은 뒤 제출하고, 접수증/제출 완료 화면을 보관합니다.</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>08_김현진_상지대_광고비지원_신청_W31_v1.pdf</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H35" s="107" t="inlineStr">
+        <is>
+          <t>공고 마감 확인 후 (초안 07-29(수))</t>
+        </is>
+      </c>
+      <c r="I35" s="47" t="inlineStr">
+        <is>
+          <t>최우선</t>
+        </is>
+      </c>
+      <c r="J35" s="114" t="n">
+        <v>8</v>
+      </c>
+      <c r="K35" s="19" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="36" ht="69" customHeight="1" s="49">
+      <c r="B36" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n"/>
-      <c r="D33" s="41" t="n"/>
-      <c r="E33" s="41" t="n"/>
-      <c r="F33" s="41" t="n"/>
-      <c r="G33" s="41" t="n"/>
-      <c r="H33" s="41" t="n"/>
-      <c r="I33" s="42" t="n"/>
-      <c r="J33" s="115">
-        <f>SUM(J28:J32)</f>
-        <v/>
-      </c>
-      <c r="K33" s="21">
-        <f>SUM(K28:K32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1" s="49">
-      <c r="B34" s="45" t="inlineStr">
+      <c r="C36" s="51" t="n"/>
+      <c r="D36" s="41" t="n"/>
+      <c r="E36" s="41" t="n"/>
+      <c r="F36" s="41" t="n"/>
+      <c r="G36" s="41" t="n"/>
+      <c r="H36" s="41" t="n"/>
+      <c r="I36" s="42" t="n"/>
+      <c r="J36" s="115">
+        <f>SUM(J28:J35)</f>
+        <v/>
+      </c>
+      <c r="K36" s="21">
+        <f>SUM(K28:K35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" s="49">
+      <c r="B37" s="45" t="inlineStr">
         <is>
           <t>발행 검증</t>
         </is>
       </c>
-      <c r="C34" s="116">
-        <f>IF(COUNTA(C28:C32)=0,"업무 미입력",IF(COUNTA(E28:E32)&lt;COUNTA(C28:C32),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F32)&lt;COUNTA(C28:C32),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K32)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K32),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
-        <v/>
-      </c>
-      <c r="D34" s="41" t="n"/>
-      <c r="E34" s="41" t="n"/>
-      <c r="F34" s="41" t="n"/>
-      <c r="G34" s="41" t="n"/>
-      <c r="H34" s="41" t="n"/>
-      <c r="I34" s="41" t="n"/>
-      <c r="J34" s="41" t="n"/>
-      <c r="K34" s="42" t="n"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" s="49"/>
-    <row r="36" ht="24" customHeight="1" s="49"/>
-    <row r="37" ht="18" customHeight="1" s="49">
-      <c r="B37" s="89" t="inlineStr">
+      <c r="C37" s="116">
+        <f>IF(COUNTA(C28:C35)=0,"업무 미입력",IF(COUNTA(E28:E35)&lt;COUNTA(C28:C35),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F35)&lt;COUNTA(C28:C35),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K35)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K35),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
+        <v/>
+      </c>
+      <c r="D37" s="41" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="41" t="n"/>
+      <c r="G37" s="41" t="n"/>
+      <c r="H37" s="41" t="n"/>
+      <c r="I37" s="41" t="n"/>
+      <c r="J37" s="41" t="n"/>
+      <c r="K37" s="42" t="n"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" s="49">
+      <c r="B38" s="45" t="n"/>
+      <c r="C38" s="117" t="n"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" s="49">
+      <c r="B39" s="45" t="n"/>
+      <c r="C39" s="118" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="49">
+      <c r="B40" s="89" t="inlineStr">
         <is>
           <t>담당자 접수확인  —  월요일 12:00까지 담당자 직접 작성 (미작성 = 업무 미이해로 간주, 재지시)</t>
         </is>
       </c>
-      <c r="C37" s="64" t="n"/>
-      <c r="D37" s="64" t="n"/>
-      <c r="E37" s="64" t="n"/>
-      <c r="F37" s="64" t="n"/>
-      <c r="G37" s="64" t="n"/>
-      <c r="H37" s="64" t="n"/>
-      <c r="I37" s="64" t="n"/>
-      <c r="J37" s="64" t="n"/>
-      <c r="K37" s="64" t="n"/>
-    </row>
-    <row r="38" ht="36" customHeight="1" s="49">
-      <c r="B38" s="45" t="inlineStr">
+      <c r="C40" s="64" t="n"/>
+      <c r="D40" s="64" t="n"/>
+      <c r="E40" s="64" t="n"/>
+      <c r="F40" s="64" t="n"/>
+      <c r="G40" s="64" t="n"/>
+      <c r="H40" s="64" t="n"/>
+      <c r="I40" s="64" t="n"/>
+      <c r="J40" s="64" t="n"/>
+      <c r="K40" s="64" t="n"/>
+    </row>
+    <row r="41" ht="36" customHeight="1" s="49">
+      <c r="B41" s="45" t="inlineStr">
         <is>
           <t>내가 이해한 업무
 (본인 언어로 재작성)</t>
         </is>
       </c>
-      <c r="C38" s="117" t="n"/>
-      <c r="D38" s="41" t="n"/>
-      <c r="E38" s="41" t="n"/>
-      <c r="F38" s="41" t="n"/>
-      <c r="G38" s="41" t="n"/>
-      <c r="H38" s="41" t="n"/>
-      <c r="I38" s="41" t="n"/>
-      <c r="J38" s="41" t="n"/>
-      <c r="K38" s="42" t="n"/>
-    </row>
-    <row r="39" ht="19.5" customHeight="1" s="49">
-      <c r="B39" s="45" t="inlineStr">
-        <is>
-          <t>완료기준 재확인
-(무엇이 되면 끝인가)</t>
-        </is>
-      </c>
-      <c r="C39" s="118" t="n"/>
-      <c r="D39" s="41" t="n"/>
-      <c r="E39" s="41" t="n"/>
-      <c r="F39" s="41" t="n"/>
-      <c r="G39" s="41" t="n"/>
-      <c r="H39" s="41" t="n"/>
-      <c r="I39" s="41" t="n"/>
-      <c r="J39" s="41" t="n"/>
-      <c r="K39" s="42" t="n"/>
-    </row>
-    <row r="40" ht="24" customHeight="1" s="49">
-      <c r="B40" s="45" t="inlineStr">
-        <is>
-          <t>예상 리스크
-(막힐 것 같은 지점)</t>
-        </is>
-      </c>
-      <c r="C40" s="43" t="n"/>
-      <c r="D40" s="41" t="n"/>
-      <c r="E40" s="41" t="n"/>
-      <c r="F40" s="41" t="n"/>
-      <c r="G40" s="41" t="n"/>
-      <c r="H40" s="41" t="n"/>
-      <c r="I40" s="41" t="n"/>
-      <c r="J40" s="41" t="n"/>
-      <c r="K40" s="42" t="n"/>
-    </row>
-    <row r="41" ht="24" customHeight="1" s="49">
-      <c r="B41" s="45" t="inlineStr">
-        <is>
-          <t>필요한 지원·의사결정</t>
-        </is>
-      </c>
-      <c r="C41" s="43" t="n"/>
+      <c r="C41" s="117" t="n"/>
       <c r="D41" s="41" t="n"/>
       <c r="E41" s="41" t="n"/>
       <c r="F41" s="41" t="n"/>
@@ -2426,13 +2530,14 @@
       <c r="J41" s="41" t="n"/>
       <c r="K41" s="42" t="n"/>
     </row>
-    <row r="42" ht="24" customHeight="1" s="49">
+    <row r="42" ht="19.5" customHeight="1" s="49">
       <c r="B42" s="45" t="inlineStr">
         <is>
-          <t>실행 계획 (요일 배분)</t>
-        </is>
-      </c>
-      <c r="C42" s="43" t="n"/>
+          <t>완료기준 재확인
+(무엇이 되면 끝인가)</t>
+        </is>
+      </c>
+      <c r="C42" s="118" t="n"/>
       <c r="D42" s="41" t="n"/>
       <c r="E42" s="41" t="n"/>
       <c r="F42" s="41" t="n"/>
@@ -2445,10 +2550,11 @@
     <row r="43" ht="24" customHeight="1" s="49">
       <c r="B43" s="45" t="inlineStr">
         <is>
-          <t>접수 확인 일시 / 서명</t>
-        </is>
-      </c>
-      <c r="C43" s="47" t="n"/>
+          <t>예상 리스크
+(막힐 것 같은 지점)</t>
+        </is>
+      </c>
+      <c r="C43" s="43" t="n"/>
       <c r="D43" s="41" t="n"/>
       <c r="E43" s="41" t="n"/>
       <c r="F43" s="41" t="n"/>
@@ -2458,14 +2564,29 @@
       <c r="J43" s="41" t="n"/>
       <c r="K43" s="42" t="n"/>
     </row>
-    <row r="44" ht="24" customHeight="1" s="49"/>
+    <row r="44" ht="24" customHeight="1" s="49">
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>필요한 지원·의사결정</t>
+        </is>
+      </c>
+      <c r="C44" s="43" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n"/>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="41" t="n"/>
+      <c r="J44" s="41" t="n"/>
+      <c r="K44" s="42" t="n"/>
+    </row>
     <row r="45" ht="24" customHeight="1" s="49">
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>결   재</t>
-        </is>
-      </c>
-      <c r="C45" s="41" t="n"/>
+      <c r="B45" s="45" t="inlineStr">
+        <is>
+          <t>실행 계획 (요일 배분)</t>
+        </is>
+      </c>
+      <c r="C45" s="43" t="n"/>
       <c r="D45" s="41" t="n"/>
       <c r="E45" s="41" t="n"/>
       <c r="F45" s="41" t="n"/>
@@ -2478,78 +2599,115 @@
     <row r="46" ht="24" customHeight="1" s="49">
       <c r="B46" s="45" t="inlineStr">
         <is>
+          <t>접수 확인 일시 / 서명</t>
+        </is>
+      </c>
+      <c r="C46" s="47" t="n"/>
+      <c r="D46" s="41" t="n"/>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+      <c r="H46" s="41" t="n"/>
+      <c r="I46" s="41" t="n"/>
+      <c r="J46" s="41" t="n"/>
+      <c r="K46" s="42" t="n"/>
+    </row>
+    <row r="47" ht="24" customHeight="1" s="49">
+      <c r="B47" s="45" t="n"/>
+      <c r="C47" s="47" t="n"/>
+      <c r="E47" s="47" t="n"/>
+      <c r="G47" s="47" t="n"/>
+      <c r="I47" s="47" t="n"/>
+      <c r="K47" s="109" t="n"/>
+    </row>
+    <row r="48" ht="24" customHeight="1" s="49">
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>결   재</t>
+        </is>
+      </c>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="41" t="n"/>
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="41" t="n"/>
+      <c r="G48" s="41" t="n"/>
+      <c r="H48" s="41" t="n"/>
+      <c r="I48" s="41" t="n"/>
+      <c r="J48" s="41" t="n"/>
+      <c r="K48" s="42" t="n"/>
+    </row>
+    <row r="49" ht="24" customHeight="1" s="49">
+      <c r="B49" s="45" t="inlineStr">
+        <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C46" s="45" t="inlineStr">
+      <c r="C49" s="45" t="inlineStr">
         <is>
           <t>작성 (지시자)</t>
         </is>
       </c>
-      <c r="D46" s="42" t="n"/>
-      <c r="E46" s="45" t="inlineStr">
+      <c r="D49" s="42" t="n"/>
+      <c r="E49" s="45" t="inlineStr">
         <is>
           <t>검토 (검수자)</t>
         </is>
       </c>
-      <c r="F46" s="42" t="n"/>
-      <c r="G46" s="45" t="inlineStr">
+      <c r="F49" s="42" t="n"/>
+      <c r="G49" s="45" t="inlineStr">
         <is>
           <t>승인 (대표)</t>
         </is>
       </c>
-      <c r="H46" s="42" t="n"/>
-      <c r="I46" s="45" t="inlineStr">
+      <c r="H49" s="42" t="n"/>
+      <c r="I49" s="45" t="inlineStr">
         <is>
           <t>접수 (담당자)</t>
         </is>
       </c>
-      <c r="J46" s="42" t="n"/>
-      <c r="K46" s="45" t="inlineStr">
+      <c r="J49" s="42" t="n"/>
+      <c r="K49" s="45" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="45" t="inlineStr">
+    <row r="50" ht="21.75" customHeight="1" s="49">
+      <c r="B50" s="45" t="inlineStr">
         <is>
           <t>서명</t>
         </is>
       </c>
-      <c r="C47" s="47" t="inlineStr">
+      <c r="C50" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="D47" s="42" t="n"/>
-      <c r="E47" s="47" t="inlineStr">
+      <c r="D50" s="42" t="n"/>
+      <c r="E50" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="F47" s="42" t="n"/>
-      <c r="G47" s="47" t="inlineStr">
+      <c r="F50" s="42" t="n"/>
+      <c r="G50" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="H47" s="42" t="n"/>
-      <c r="I47" s="47" t="inlineStr">
+      <c r="H50" s="42" t="n"/>
+      <c r="I50" s="47" t="inlineStr">
         <is>
           <t>김 현 진</t>
         </is>
       </c>
-      <c r="J47" s="42" t="n"/>
-      <c r="K47" s="109" t="inlineStr">
+      <c r="J50" s="42" t="n"/>
+      <c r="K50" s="109" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="19.5" customHeight="1" s="49"/>
-    <row r="49" ht="21.75" customHeight="1" s="49"/>
-    <row r="50" ht="21.75" customHeight="1" s="49"/>
     <row r="51" ht="21.75" customHeight="1" s="49"/>
     <row r="52" ht="21.75" customHeight="1" s="49"/>
     <row r="53" ht="21.75" customHeight="1" s="49"/>
@@ -2568,48 +2726,48 @@
     <row r="68" ht="39.75" customHeight="1" s="49"/>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="C41:K41"/>
     <mergeCell ref="C10:K10"/>
-    <mergeCell ref="C41:K41"/>
+    <mergeCell ref="B40:K40"/>
     <mergeCell ref="C15:J15"/>
-    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="C44:K44"/>
     <mergeCell ref="C24:J24"/>
-    <mergeCell ref="C40:K40"/>
+    <mergeCell ref="I49:J49"/>
     <mergeCell ref="C9:K9"/>
     <mergeCell ref="C14:J14"/>
     <mergeCell ref="C43:K43"/>
-    <mergeCell ref="B45:K45"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="C46:K46"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="B26:K26"/>
     <mergeCell ref="C16:J16"/>
+    <mergeCell ref="C50:D50"/>
     <mergeCell ref="B7:K7"/>
-    <mergeCell ref="C39:K39"/>
+    <mergeCell ref="C22:J22"/>
     <mergeCell ref="C8:K8"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="C33:I33"/>
     <mergeCell ref="B14:B21"/>
-    <mergeCell ref="C38:K38"/>
-    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="G49:H49"/>
     <mergeCell ref="C21:J21"/>
-    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C37:K37"/>
+    <mergeCell ref="E49:F49"/>
     <mergeCell ref="B12:K12"/>
+    <mergeCell ref="B48:K48"/>
     <mergeCell ref="B2:K2"/>
-    <mergeCell ref="C34:K34"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="C17:J17"/>
     <mergeCell ref="B1:K1"/>
-    <mergeCell ref="G47:H47"/>
     <mergeCell ref="C42:K42"/>
-    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="C45:K45"/>
     <mergeCell ref="C19:J19"/>
+    <mergeCell ref="I50:J50"/>
     <mergeCell ref="C13:J13"/>
+    <mergeCell ref="C49:D49"/>
     <mergeCell ref="C18:J18"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="B37:K37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I28:I32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I28:I35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"최우선,높음,보통,낮음"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2624,7 +2782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:L47"/>
+  <dimension ref="C1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="19.85546875" customWidth="1" style="49" min="3" max="3"/>
@@ -2705,7 +2863,7 @@
         </is>
       </c>
       <c r="D5" s="26">
-        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
+        <f>SUMPRODUCT(F12:F19,H12:H19)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2723,7 +2881,7 @@
         </is>
       </c>
       <c r="H5" s="119">
-        <f>SUM('01_업무지시서'!J28:J32)</f>
+        <f>SUM('01_업무지시서'!J28:J35)</f>
         <v/>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -2732,7 +2890,7 @@
         </is>
       </c>
       <c r="J5" s="119">
-        <f>SUM(I12:I16)</f>
+        <f>SUM(I12:I19)</f>
         <v/>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -3014,133 +3172,160 @@
       <c r="K16" s="47" t="n"/>
       <c r="L16" s="47" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1" s="49">
-      <c r="C17" s="45" t="inlineStr">
+    <row r="17" ht="27.75" customHeight="1" s="49">
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="40">
+        <f>IF('01_업무지시서'!C33="","",'01_업무지시서'!C33)</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>IF('01_업무지시서'!E33="","",'01_업무지시서'!E33)</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
+        <f>IF('01_업무지시서'!K33="",0,'01_업무지시서'!K33)</f>
+        <v/>
+      </c>
+      <c r="G17" s="47" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="114" t="n"/>
+      <c r="J17" s="47" t="n"/>
+      <c r="K17" s="47" t="n"/>
+      <c r="L17" s="47" t="n"/>
+    </row>
+    <row r="18" ht="27.75" customHeight="1" s="49">
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="40">
+        <f>IF('01_업무지시서'!C34="","",'01_업무지시서'!C34)</f>
+        <v/>
+      </c>
+      <c r="E18" s="40">
+        <f>IF('01_업무지시서'!E34="","",'01_업무지시서'!E34)</f>
+        <v/>
+      </c>
+      <c r="F18" s="11">
+        <f>IF('01_업무지시서'!K34="",0,'01_업무지시서'!K34)</f>
+        <v/>
+      </c>
+      <c r="G18" s="47" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="114" t="n"/>
+      <c r="J18" s="47" t="n"/>
+      <c r="K18" s="47" t="n"/>
+      <c r="L18" s="47" t="n"/>
+    </row>
+    <row r="19" ht="27.75" customHeight="1" s="49">
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="40">
+        <f>IF('01_업무지시서'!C35="","",'01_업무지시서'!C35)</f>
+        <v/>
+      </c>
+      <c r="E19" s="40">
+        <f>IF('01_업무지시서'!E35="","",'01_업무지시서'!E35)</f>
+        <v/>
+      </c>
+      <c r="F19" s="11">
+        <f>IF('01_업무지시서'!K35="",0,'01_업무지시서'!K35)</f>
+        <v/>
+      </c>
+      <c r="G19" s="47" t="n"/>
+      <c r="H19" s="19" t="n"/>
+      <c r="I19" s="114" t="n"/>
+      <c r="J19" s="47" t="n"/>
+      <c r="K19" s="47" t="n"/>
+      <c r="L19" s="47" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="49">
+      <c r="C20" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D17" s="45" t="inlineStr">
+      <c r="D20" s="45" t="inlineStr">
         <is>
           <t>가중 달성률 →</t>
         </is>
       </c>
-      <c r="E17" s="42" t="n"/>
-      <c r="F17" s="21">
-        <f>SUM(F12:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="28">
-        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="29">
-        <f>COUNTIF(G12:G16,"완료")</f>
-        <v/>
-      </c>
-      <c r="I17" s="115">
-        <f>SUM(I12:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="69">
-        <f>"완료 "&amp;COUNTIF(G12:G16,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G16,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G16,"미착수")&amp;"건"</f>
-        <v/>
-      </c>
-      <c r="K17" s="41" t="n"/>
-      <c r="L17" s="42" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1" s="49">
-      <c r="C18" s="46" t="n"/>
-      <c r="D18" s="46" t="n"/>
-      <c r="I18" s="46" t="n"/>
-      <c r="J18" s="46" t="n"/>
-      <c r="L18" s="46" t="n"/>
-    </row>
-    <row r="19" ht="19.5" customHeight="1" s="49">
-      <c r="C19" s="121" t="inlineStr">
+      <c r="E20" s="42" t="n"/>
+      <c r="F20" s="21">
+        <f>SUM(F12:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="28">
+        <f>SUMPRODUCT(F12:F19,H12:H19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="29">
+        <f>COUNTIF(G12:G19,"완료")</f>
+        <v/>
+      </c>
+      <c r="I20" s="115">
+        <f>SUM(I12:I19)</f>
+        <v/>
+      </c>
+      <c r="J20" s="69">
+        <f>"완료 "&amp;COUNTIF(G12:G19,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G19,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G19,"미착수")&amp;"건"</f>
+        <v/>
+      </c>
+      <c r="K20" s="41" t="n"/>
+      <c r="L20" s="42" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1" s="49">
+      <c r="C21" s="46" t="n"/>
+      <c r="D21" s="46" t="n"/>
+      <c r="I21" s="46" t="n"/>
+      <c r="J21" s="46" t="n"/>
+      <c r="L21" s="46" t="n"/>
+    </row>
+    <row r="22" ht="19.5" customHeight="1" s="49">
+      <c r="C22" s="121" t="inlineStr">
         <is>
           <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
         </is>
       </c>
-      <c r="D19" s="64" t="n"/>
-      <c r="E19" s="64" t="n"/>
-      <c r="F19" s="64" t="n"/>
-      <c r="G19" s="64" t="n"/>
-      <c r="H19" s="64" t="n"/>
-      <c r="I19" s="64" t="n"/>
-      <c r="J19" s="64" t="n"/>
-      <c r="K19" s="64" t="n"/>
-      <c r="L19" s="65" t="n"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" s="49">
-      <c r="C20" s="46" t="inlineStr">
+      <c r="D22" s="64" t="n"/>
+      <c r="E22" s="64" t="n"/>
+      <c r="F22" s="64" t="n"/>
+      <c r="G22" s="64" t="n"/>
+      <c r="H22" s="64" t="n"/>
+      <c r="I22" s="64" t="n"/>
+      <c r="J22" s="64" t="n"/>
+      <c r="K22" s="64" t="n"/>
+      <c r="L22" s="65" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="49">
+      <c r="C23" s="46" t="inlineStr">
         <is>
           <t>검수 항목 (자동)</t>
         </is>
       </c>
-      <c r="D20" s="46" t="inlineStr">
+      <c r="D23" s="46" t="inlineStr">
         <is>
           <t>검수 질문 (자동)</t>
         </is>
       </c>
-      <c r="E20" s="41" t="n"/>
-      <c r="F20" s="41" t="n"/>
-      <c r="G20" s="41" t="n"/>
-      <c r="H20" s="42" t="n"/>
-      <c r="I20" s="46" t="inlineStr">
-        <is>
-          <t>자가
-판정</t>
-        </is>
-      </c>
-      <c r="J20" s="46" t="inlineStr">
-        <is>
-          <t>미충족 사유·보완 계획</t>
-        </is>
-      </c>
-      <c r="K20" s="42" t="n"/>
-      <c r="L20" s="46" t="inlineStr">
-        <is>
-          <t>검수자
-판정</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1" s="49">
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="55" t="n"/>
-      <c r="E21" s="41" t="n"/>
-      <c r="F21" s="41" t="n"/>
-      <c r="G21" s="41" t="n"/>
-      <c r="H21" s="42" t="n"/>
-      <c r="I21" s="47" t="n"/>
-      <c r="J21" s="44" t="n"/>
-      <c r="K21" s="42" t="n"/>
-      <c r="L21" s="66" t="n"/>
-    </row>
-    <row r="22" ht="24" customHeight="1" s="49">
-      <c r="C22" s="69" t="n"/>
-      <c r="D22" s="55" t="n"/>
-      <c r="E22" s="41" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="42" t="n"/>
-      <c r="I22" s="47" t="n"/>
-      <c r="J22" s="44" t="n"/>
-      <c r="K22" s="42" t="n"/>
-      <c r="L22" s="66" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1" s="49">
-      <c r="C23" s="69" t="n"/>
-      <c r="D23" s="55" t="n"/>
       <c r="E23" s="41" t="n"/>
       <c r="F23" s="41" t="n"/>
       <c r="G23" s="41" t="n"/>
       <c r="H23" s="42" t="n"/>
-      <c r="I23" s="47" t="n"/>
-      <c r="J23" s="44" t="n"/>
+      <c r="I23" s="46" t="inlineStr">
+        <is>
+          <t>자가
+판정</t>
+        </is>
+      </c>
+      <c r="J23" s="46" t="inlineStr">
+        <is>
+          <t>미충족 사유·보완 계획</t>
+        </is>
+      </c>
       <c r="K23" s="42" t="n"/>
-      <c r="L23" s="66" t="n"/>
+      <c r="L23" s="46" t="inlineStr">
+        <is>
+          <t>검수자
+판정</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="24" customHeight="1" s="49">
       <c r="C24" s="69" t="n"/>
@@ -3190,249 +3375,243 @@
       <c r="K27" s="42" t="n"/>
       <c r="L27" s="66" t="n"/>
     </row>
-    <row r="28" ht="27.75" customHeight="1" s="49">
-      <c r="C28" s="46" t="n"/>
-      <c r="D28" s="46" t="n"/>
-      <c r="E28" s="46" t="n"/>
-      <c r="F28" s="46" t="n"/>
-      <c r="G28" s="46" t="n"/>
-      <c r="H28" s="46" t="n"/>
-      <c r="I28" s="46" t="n"/>
-      <c r="J28" s="46" t="n"/>
-      <c r="K28" s="46" t="n"/>
-      <c r="L28" s="46" t="n"/>
-    </row>
-    <row r="29" ht="19.5" customHeight="1" s="49">
-      <c r="C29" s="121" t="inlineStr">
+    <row r="28" ht="24" customHeight="1" s="49">
+      <c r="C28" s="69" t="n"/>
+      <c r="D28" s="55" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="41" t="n"/>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="47" t="n"/>
+      <c r="J28" s="44" t="n"/>
+      <c r="K28" s="42" t="n"/>
+      <c r="L28" s="66" t="n"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" s="49">
+      <c r="C29" s="69" t="n"/>
+      <c r="D29" s="55" t="n"/>
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="41" t="n"/>
+      <c r="G29" s="41" t="n"/>
+      <c r="H29" s="42" t="n"/>
+      <c r="I29" s="47" t="n"/>
+      <c r="J29" s="44" t="n"/>
+      <c r="K29" s="42" t="n"/>
+      <c r="L29" s="66" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" s="49">
+      <c r="C30" s="69" t="n"/>
+      <c r="D30" s="55" t="n"/>
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="41" t="n"/>
+      <c r="G30" s="41" t="n"/>
+      <c r="H30" s="42" t="n"/>
+      <c r="I30" s="47" t="n"/>
+      <c r="J30" s="44" t="n"/>
+      <c r="K30" s="42" t="n"/>
+      <c r="L30" s="66" t="n"/>
+    </row>
+    <row r="31" ht="27.75" customHeight="1" s="49">
+      <c r="C31" s="46" t="n"/>
+      <c r="D31" s="46" t="n"/>
+      <c r="E31" s="46" t="n"/>
+      <c r="F31" s="46" t="n"/>
+      <c r="G31" s="46" t="n"/>
+      <c r="H31" s="46" t="n"/>
+      <c r="I31" s="46" t="n"/>
+      <c r="J31" s="46" t="n"/>
+      <c r="K31" s="46" t="n"/>
+      <c r="L31" s="46" t="n"/>
+    </row>
+    <row r="32" ht="19.5" customHeight="1" s="49">
+      <c r="C32" s="121" t="inlineStr">
         <is>
           <t>3. 이슈 및 지원요청  —  대안 없이 문제만 올리는 보고는 반려</t>
         </is>
       </c>
-      <c r="D29" s="64" t="n"/>
-      <c r="E29" s="64" t="n"/>
-      <c r="F29" s="64" t="n"/>
-      <c r="G29" s="64" t="n"/>
-      <c r="H29" s="64" t="n"/>
-      <c r="I29" s="64" t="n"/>
-      <c r="J29" s="64" t="n"/>
-      <c r="K29" s="64" t="n"/>
-      <c r="L29" s="65" t="n"/>
-    </row>
-    <row r="30" ht="27.75" customHeight="1" s="49">
-      <c r="C30" s="46" t="inlineStr">
+      <c r="D32" s="64" t="n"/>
+      <c r="E32" s="64" t="n"/>
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="64" t="n"/>
+      <c r="H32" s="64" t="n"/>
+      <c r="I32" s="64" t="n"/>
+      <c r="J32" s="64" t="n"/>
+      <c r="K32" s="64" t="n"/>
+      <c r="L32" s="65" t="n"/>
+    </row>
+    <row r="33" ht="27.75" customHeight="1" s="49">
+      <c r="C33" s="46" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D30" s="46" t="inlineStr">
+      <c r="D33" s="46" t="inlineStr">
         <is>
           <t>이슈 내용</t>
         </is>
       </c>
-      <c r="E30" s="46" t="inlineStr">
+      <c r="E33" s="46" t="inlineStr">
         <is>
           <t>영향
 (일정/비용/품질)</t>
         </is>
       </c>
-      <c r="F30" s="46" t="inlineStr">
+      <c r="F33" s="46" t="inlineStr">
         <is>
           <t>근본 원인</t>
         </is>
       </c>
-      <c r="G30" s="46" t="inlineStr">
+      <c r="G33" s="46" t="inlineStr">
         <is>
           <t>대안 1</t>
         </is>
       </c>
-      <c r="H30" s="46" t="inlineStr">
+      <c r="H33" s="46" t="inlineStr">
         <is>
           <t>대안 2</t>
         </is>
       </c>
-      <c r="I30" s="46" t="inlineStr">
+      <c r="I33" s="46" t="inlineStr">
         <is>
           <t>권고안</t>
         </is>
       </c>
-      <c r="J30" s="46" t="inlineStr">
+      <c r="J33" s="46" t="inlineStr">
         <is>
           <t>요청사항</t>
         </is>
       </c>
-      <c r="K30" s="46" t="inlineStr">
+      <c r="K33" s="46" t="inlineStr">
         <is>
           <t>결정기한</t>
         </is>
       </c>
-      <c r="L30" s="46" t="inlineStr">
+      <c r="L33" s="46" t="inlineStr">
         <is>
           <t>대표 결정</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1" s="49">
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="66" t="n"/>
-    </row>
-    <row r="32" ht="36" customHeight="1" s="49">
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="66" t="n"/>
-    </row>
-    <row r="33" ht="36" customHeight="1" s="49">
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="18" t="n"/>
-      <c r="J33" s="18" t="n"/>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="66" t="n"/>
-    </row>
-    <row r="34" ht="27.75" customHeight="1" s="49">
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="46" t="n"/>
-      <c r="E34" s="46" t="n"/>
-      <c r="F34" s="46" t="n"/>
-      <c r="G34" s="46" t="n"/>
-      <c r="H34" s="46" t="n"/>
-      <c r="I34" s="46" t="n"/>
-      <c r="J34" s="46" t="n"/>
-      <c r="K34" s="46" t="n"/>
-      <c r="L34" s="46" t="n"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1" s="49">
-      <c r="C35" s="121" t="inlineStr">
+    <row r="34" ht="36" customHeight="1" s="49">
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="18" t="n"/>
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="66" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1" s="49">
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="18" t="n"/>
+      <c r="J35" s="18" t="n"/>
+      <c r="K35" s="6" t="n"/>
+      <c r="L35" s="66" t="n"/>
+    </row>
+    <row r="36" ht="36" customHeight="1" s="49">
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="18" t="n"/>
+      <c r="J36" s="18" t="n"/>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="66" t="n"/>
+    </row>
+    <row r="37" ht="27.75" customHeight="1" s="49">
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="46" t="n"/>
+      <c r="E37" s="46" t="n"/>
+      <c r="F37" s="46" t="n"/>
+      <c r="G37" s="46" t="n"/>
+      <c r="H37" s="46" t="n"/>
+      <c r="I37" s="46" t="n"/>
+      <c r="J37" s="46" t="n"/>
+      <c r="K37" s="46" t="n"/>
+      <c r="L37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="19.5" customHeight="1" s="49">
+      <c r="C38" s="121" t="inlineStr">
         <is>
           <t>4. 다음 주 제안 업무  —  지시를 기다리지 말 것. 본인이 먼저 제안.</t>
         </is>
       </c>
-      <c r="D35" s="64" t="n"/>
-      <c r="E35" s="64" t="n"/>
-      <c r="F35" s="64" t="n"/>
-      <c r="G35" s="64" t="n"/>
-      <c r="H35" s="64" t="n"/>
-      <c r="I35" s="64" t="n"/>
-      <c r="J35" s="64" t="n"/>
-      <c r="K35" s="64" t="n"/>
-      <c r="L35" s="65" t="n"/>
-    </row>
-    <row r="36" ht="27.75" customHeight="1" s="49">
-      <c r="C36" s="13" t="inlineStr">
+      <c r="D38" s="64" t="n"/>
+      <c r="E38" s="64" t="n"/>
+      <c r="F38" s="64" t="n"/>
+      <c r="G38" s="64" t="n"/>
+      <c r="H38" s="64" t="n"/>
+      <c r="I38" s="64" t="n"/>
+      <c r="J38" s="64" t="n"/>
+      <c r="K38" s="64" t="n"/>
+      <c r="L38" s="65" t="n"/>
+    </row>
+    <row r="39" ht="27.75" customHeight="1" s="49">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D36" s="46" t="inlineStr">
+      <c r="D39" s="46" t="inlineStr">
         <is>
           <t>제안 업무</t>
         </is>
       </c>
-      <c r="E36" s="46" t="inlineStr">
+      <c r="E39" s="46" t="inlineStr">
         <is>
           <t>왜 해야 하는가</t>
         </is>
       </c>
-      <c r="F36" s="46" t="inlineStr">
+      <c r="F39" s="46" t="inlineStr">
         <is>
           <t>완료기준(안)</t>
         </is>
       </c>
-      <c r="G36" s="46" t="inlineStr">
+      <c r="G39" s="46" t="inlineStr">
         <is>
           <t>예상
 소요(h)</t>
         </is>
       </c>
-      <c r="H36" s="46" t="inlineStr">
+      <c r="H39" s="46" t="inlineStr">
         <is>
           <t>우선순위(안)</t>
         </is>
       </c>
-      <c r="I36" s="46" t="inlineStr">
+      <c r="I39" s="46" t="inlineStr">
         <is>
           <t>선행 조건</t>
         </is>
       </c>
-      <c r="J36" s="46" t="inlineStr">
+      <c r="J39" s="46" t="inlineStr">
         <is>
           <t>필요 지원</t>
         </is>
       </c>
-      <c r="K36" s="46" t="inlineStr">
+      <c r="K39" s="46" t="inlineStr">
         <is>
           <t>대표 승인</t>
         </is>
       </c>
-      <c r="L36" s="46" t="inlineStr">
+      <c r="L39" s="46" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="31.5" customHeight="1" s="49">
-      <c r="C37" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="114" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="66" t="n"/>
-      <c r="L37" s="6" t="n"/>
-    </row>
-    <row r="38" ht="31.5" customHeight="1" s="49">
-      <c r="C38" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="114" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
-      <c r="K38" s="66" t="n"/>
-      <c r="L38" s="6" t="n"/>
-    </row>
-    <row r="39" ht="31.5" customHeight="1" s="49">
-      <c r="C39" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="114" t="n"/>
-      <c r="H39" s="6" t="n"/>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
-      <c r="K39" s="66" t="n"/>
-      <c r="L39" s="6" t="n"/>
     </row>
     <row r="40" ht="31.5" customHeight="1" s="49">
       <c r="C40" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D40" s="18" t="n"/>
       <c r="E40" s="18" t="n"/>
@@ -3444,136 +3623,178 @@
       <c r="K40" s="66" t="n"/>
       <c r="L40" s="6" t="n"/>
     </row>
-    <row r="41" ht="25.5" customHeight="1" s="49">
-      <c r="C41" s="45" t="n"/>
-      <c r="D41" s="43" t="n"/>
-      <c r="J41" s="58" t="n"/>
-    </row>
-    <row r="42" ht="19.5" customHeight="1" s="49">
-      <c r="C42" s="48" t="inlineStr">
+    <row r="41" ht="31.5" customHeight="1" s="49">
+      <c r="C41" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="114" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="66" t="n"/>
+      <c r="L41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="31.5" customHeight="1" s="49">
+      <c r="C42" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="18" t="n"/>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="114" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="18" t="n"/>
+      <c r="K42" s="66" t="n"/>
+      <c r="L42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="31.5" customHeight="1" s="49">
+      <c r="C43" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="114" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="18" t="n"/>
+      <c r="J43" s="18" t="n"/>
+      <c r="K43" s="66" t="n"/>
+      <c r="L43" s="6" t="n"/>
+    </row>
+    <row r="44" ht="25.5" customHeight="1" s="49">
+      <c r="C44" s="45" t="n"/>
+      <c r="D44" s="43" t="n"/>
+      <c r="J44" s="58" t="n"/>
+    </row>
+    <row r="45" ht="19.5" customHeight="1" s="49">
+      <c r="C45" s="48" t="inlineStr">
         <is>
           <t>5. 자기점검 및 대표 검수</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="25.5" customHeight="1" s="49">
-      <c r="C43" s="45" t="inlineStr">
+    <row r="46" ht="25.5" customHeight="1" s="49">
+      <c r="C46" s="45" t="inlineStr">
         <is>
           <t>이번 주 가장 잘한 것</t>
         </is>
       </c>
-      <c r="D43" s="43" t="inlineStr">
+      <c r="D46" s="43" t="inlineStr">
         <is>
           <t>결과로 증명되는 것 1개만</t>
         </is>
       </c>
-      <c r="E43" s="41" t="n"/>
-      <c r="F43" s="41" t="n"/>
-      <c r="G43" s="41" t="n"/>
-      <c r="H43" s="41" t="n"/>
-      <c r="I43" s="42" t="n"/>
-      <c r="J43" s="58" t="inlineStr">
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+      <c r="H46" s="41" t="n"/>
+      <c r="I46" s="42" t="n"/>
+      <c r="J46" s="58" t="inlineStr">
         <is>
           <t>[대표 검수 의견]</t>
         </is>
       </c>
-      <c r="K43" s="59" t="n"/>
-      <c r="L43" s="60" t="n"/>
-    </row>
-    <row r="44" ht="25.5" customHeight="1" s="49">
-      <c r="C44" s="45" t="inlineStr">
+      <c r="K46" s="59" t="n"/>
+      <c r="L46" s="60" t="n"/>
+    </row>
+    <row r="47" ht="25.5" customHeight="1" s="49">
+      <c r="C47" s="45" t="inlineStr">
         <is>
           <t>이번 주 가장 부족한 것</t>
         </is>
       </c>
-      <c r="D44" s="43" t="inlineStr">
+      <c r="D47" s="43" t="inlineStr">
         <is>
           <t>변명 말고 사실만</t>
         </is>
       </c>
-      <c r="E44" s="41" t="n"/>
-      <c r="F44" s="41" t="n"/>
-      <c r="G44" s="41" t="n"/>
-      <c r="H44" s="41" t="n"/>
-      <c r="I44" s="42" t="n"/>
-      <c r="J44" s="61" t="n"/>
-      <c r="L44" s="62" t="n"/>
-    </row>
-    <row r="45" ht="25.5" customHeight="1" s="49">
-      <c r="C45" s="45" t="inlineStr">
+      <c r="E47" s="41" t="n"/>
+      <c r="F47" s="41" t="n"/>
+      <c r="G47" s="41" t="n"/>
+      <c r="H47" s="41" t="n"/>
+      <c r="I47" s="42" t="n"/>
+      <c r="J47" s="61" t="n"/>
+      <c r="L47" s="62" t="n"/>
+    </row>
+    <row r="48" ht="25.5" customHeight="1" s="49">
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>다음 주 개선 액션 1개</t>
         </is>
       </c>
-      <c r="D45" s="43" t="inlineStr">
+      <c r="D48" s="43" t="inlineStr">
         <is>
           <t>실행 가능한 행동으로</t>
         </is>
       </c>
-      <c r="E45" s="41" t="n"/>
-      <c r="F45" s="41" t="n"/>
-      <c r="G45" s="41" t="n"/>
-      <c r="H45" s="41" t="n"/>
-      <c r="I45" s="42" t="n"/>
-      <c r="J45" s="63" t="n"/>
-      <c r="K45" s="64" t="n"/>
-      <c r="L45" s="65" t="n"/>
-    </row>
-    <row r="47" ht="33.75" customHeight="1" s="49">
-      <c r="C47" s="45" t="inlineStr">
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="41" t="n"/>
+      <c r="G48" s="41" t="n"/>
+      <c r="H48" s="41" t="n"/>
+      <c r="I48" s="42" t="n"/>
+      <c r="J48" s="63" t="n"/>
+      <c r="K48" s="64" t="n"/>
+      <c r="L48" s="65" t="n"/>
+    </row>
+    <row r="50" ht="33.75" customHeight="1" s="49">
+      <c r="C50" s="45" t="inlineStr">
         <is>
           <t>제출자</t>
         </is>
       </c>
-      <c r="D47" s="47" t="n"/>
-      <c r="E47" s="41" t="n"/>
-      <c r="F47" s="42" t="n"/>
-      <c r="G47" s="45" t="inlineStr">
+      <c r="D50" s="47" t="n"/>
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="42" t="n"/>
+      <c r="G50" s="45" t="inlineStr">
         <is>
           <t>검수자</t>
         </is>
       </c>
-      <c r="H47" s="66" t="n"/>
-      <c r="I47" s="42" t="n"/>
-      <c r="J47" s="45" t="inlineStr">
+      <c r="H50" s="66" t="n"/>
+      <c r="I50" s="42" t="n"/>
+      <c r="J50" s="45" t="inlineStr">
         <is>
           <t>최종 판정</t>
         </is>
       </c>
-      <c r="K47" s="56" t="n"/>
-      <c r="L47" s="42" t="n"/>
+      <c r="K50" s="56" t="n"/>
+      <c r="L50" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="C32:L32"/>
+    <mergeCell ref="C38:L38"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="D48:I48"/>
+    <mergeCell ref="D47:I47"/>
     <mergeCell ref="D7:L7"/>
-    <mergeCell ref="D43:I43"/>
-    <mergeCell ref="C19:L19"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="J24:K24"/>
+    <mergeCell ref="K50:L50"/>
     <mergeCell ref="D27:H27"/>
     <mergeCell ref="J27:K27"/>
-    <mergeCell ref="C42:L42"/>
-    <mergeCell ref="D17:E17"/>
     <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="C45:L45"/>
+    <mergeCell ref="J46:L48"/>
     <mergeCell ref="J25:K25"/>
-    <mergeCell ref="C29:L29"/>
-    <mergeCell ref="C35:L35"/>
-    <mergeCell ref="J43:L45"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="D44:I44"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="D50:F50"/>
     <mergeCell ref="C1:L1"/>
-    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D30:H30"/>
     <mergeCell ref="D25:H25"/>
+    <mergeCell ref="C22:L22"/>
+    <mergeCell ref="D46:I46"/>
     <mergeCell ref="C9:L9"/>
     <mergeCell ref="D24:H24"/>
-    <mergeCell ref="D45:I45"/>
+    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D23:H23"/>
     <mergeCell ref="J23:K23"/>
     <mergeCell ref="C2:L2"/>
@@ -3581,19 +3802,19 @@
     <mergeCell ref="D26:H26"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="I21:I27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I24:I30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"충족,미충족"</formula1>
     </dataValidation>
-    <dataValidation sqref="L21:L27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L24:L30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,보완,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="K37:K40 L31:L33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K40:K43 L34:L36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"승인,보류,반려"</formula1>
     </dataValidation>
-    <dataValidation sqref="K47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,조건부합격,보완요청,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="G12:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G12:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행중,미착수,보류,취소"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Revise 김현진 W31: CRM-centric with monthly report, call-center, AI automation
Fold operations process into CRM as productized entries; add CRM monthly-
report generation; split consultation into a separate call-center response
build; convert pipeline tracking to AI automation; drop partner sales.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_김현진_2026-W31.xlsx
+++ b/out/BRING_주간_김현진_2026-W31.xlsx
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E5" s="110" t="inlineStr">
         <is>
-          <t>운영관리팀장 / 입·퇴실 패키지 영업 관리</t>
+          <t>운영관리팀장 / 입·퇴실 패키지·CRM 관리</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
@@ -1693,9 +1693,8 @@
       </c>
       <c r="C8" s="70" t="inlineStr">
         <is>
-          <t>김현진 팀장은 입·퇴실 패키지 상품화부터 고객 상담·견적·계약까지 영업 전 과정을 관리합니다. 추가로 상지대학교 광고비 100만 원 지원금 신청서 작성 및 제출 준비를 담당합니다.
-지금은 입·퇴실 패키지가 '판매 가능한 상품'으로 정리되어 있지 않고 고객 문의가 체계적으로 관리되지 않습니다. 이번 주에는 패키지를 바로 설명·판매할 수 있는 형태로 완성하고, CRM으로 문의부터 상담·견적·계약까지 관리하는 기반을 만들며, 마감이 있는 상지대 광고비 지원 신청을 준비합니다.
-한 문장으로: 입·퇴실 패키지를 판매 가능한 상품으로 완성하고, CRM으로 문의~계약을 관리하며, 잠재고객·제휴처 영업과 상지대 광고비 지원 신청을 담당합니다.</t>
+          <t>김현진 팀장은 입·퇴실 패키지 상품화부터 고객 상담·견적·계약까지 영업 전 과정을 'CRM 안에서' 이뤄지도록 구축·관리합니다. 우리가 정리해 둔 운영 프로세스는 상품정의서·소개서·상담문구·가격표 같은 '상품화 형태'로 더 세분화해 CRM에 반영합니다.
+또한 CRM에 쌓인 데이터를 매달 '월간보고서'로 받아볼 수 있게 만들고, 고객 상담 대응은 고객센터용으로 별도 구축하며(CRM·마케팅·고객센터 3축), 문의~계약 진행상황 점검은 사람이 매일 수기로 하지 않고 AI 자동화로 처리되게 합니다. 추가로 마감이 있는 상지대 광고비 100만 원 지원 신청을 준비합니다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1716,7 +1715,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>입·퇴실 패키지를 바로 판매·설명할 수 있는 상품으로 완성하고, CRM으로 문의~상담~견적~계약을 관리하며, 상지대 광고비 100만 원 지원 신청서를 준비하는 것입니다.</t>
+          <t>입·퇴실 패키지와 운영 프로세스를 상품화해 CRM에 반영하고, 상담·견적·계약·사후관리가 CRM 안에서 이뤄지게 하며, 월간보고서 자동 산출·고객센터 대응 구축·진행상황 AI 자동화·상지대 지원 신청을 진행합니다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1737,7 +1736,7 @@
       </c>
       <c r="C10" s="73" t="inlineStr">
         <is>
-          <t>패키지가 상품으로 정리되지 않으면 문의가 와도 즉시 판매·견적이 어렵고, CRM 없이 관리하면 상담·견적·재연락이 누락됩니다. 또한 상지대 광고비 지원은 마감이 있어 준비가 늦으면 100만 원 지원 기회를 놓칩니다.</t>
+          <t>패키지·프로세스가 CRM에 상품화되어 반영되지 않으면 문의가 와도 즉시 판매·견적이 어렵고, CRM·월간보고서가 없으면 상담·견적·재연락이 누락되고 월 단위 성과를 파악할 수 없습니다. 상지대 광고비 지원은 마감이 있어 늦으면 100만 원 기회를 놓칩니다.</t>
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
@@ -1788,7 +1787,7 @@
       </c>
       <c r="C14" s="111" t="inlineStr">
         <is>
-          <t>1. 입·퇴실 패키지 상품화 (상품정의서·고객용 소개서·상담문구·가격/옵션표)</t>
+          <t>1. 입·퇴실 패키지 상품화 (상품정의서·소개서·상담문구·가격표)</t>
         </is>
       </c>
       <c r="D14" s="41" t="n"/>
@@ -1808,7 +1807,7 @@
       <c r="B15" s="112" t="n"/>
       <c r="C15" s="111" t="inlineStr">
         <is>
-          <t>2. CRM 구축·관리 (진행 14단계·필수 입력정보·관리 기준 적용)</t>
+          <t>2. CRM 구축·관리 — 운영 프로세스를 상품화 형태로 세분화해 CRM에 반영 (모든 업무가 CRM 안에서)</t>
         </is>
       </c>
       <c r="D15" s="41" t="n"/>
@@ -1824,7 +1823,7 @@
       <c r="B16" s="112" t="n"/>
       <c r="C16" s="111" t="inlineStr">
         <is>
-          <t>3. 고객 상담 (확인사항·상담 후 처리·상담 문구 세트)</t>
+          <t>3. 고객센터용 상담 대응 페이지 별도 구축 (CRM·마케팅과 구분되는 고객센터 축)</t>
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
@@ -1840,7 +1839,7 @@
       <c r="B17" s="112" t="n"/>
       <c r="C17" s="111" t="inlineStr">
         <is>
-          <t>4. 견적 및 계약 진행 (견적 전 확인·발송 후 관리·계약 확정 절차)</t>
+          <t>4. 견적·계약 진행 정비 (CRM 내에서 연결)</t>
         </is>
       </c>
       <c r="D17" s="41" t="n"/>
@@ -1856,7 +1855,7 @@
       <c r="B18" s="112" t="n"/>
       <c r="C18" s="111" t="inlineStr">
         <is>
-          <t>5. 잠재고객·제휴처 영업 (대상·기록항목·제안내용)</t>
+          <t>5. 문의~계약 진행상황 관리 AI 자동화 (매일 점검·지연고객 알림)</t>
         </is>
       </c>
       <c r="D18" s="41" t="n"/>
@@ -1872,7 +1871,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>6. 문의~계약 전체 진행상황 관리 (매일 점검·지연고객 관리)</t>
+          <t>6. CRM 월간보고서 자동 산출 기능 만들기</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1924,12 +1923,12 @@
       </c>
       <c r="C22" s="105" t="inlineStr">
         <is>
-          <t>대표 확인/승인 후에만 진행:
+          <t>· 잠재고객·제휴처 영업은 이번 주 범위에서 제외
+대표 확인/승인 후에만 진행:
 · 가격 변경·할인 (견적 가격 변경은 대표 승인 후)
-· 제휴 조건·소개 수수료 확정
 · 외부 기관(상지대 등) 최종 제출
 · 개인정보 포함 자료의 공개 링크 사용 (금지)
-· 계약 실패 고객 정보 삭제 (삭제 금지 — 실패 이유 기록)</t>
+· 계약 실패 고객 정보 삭제 (금지 — 실패 이유 기록)</t>
         </is>
       </c>
       <c r="D22" s="41" t="n"/>
@@ -1953,10 +1952,11 @@
       </c>
       <c r="C23" s="105" t="inlineStr">
         <is>
-          <t>· 모든 고객에게 반드시 3가지: ① 현재 진행상태 ② 담당자 ③ 다음 행동·예정일
-· 신규 문의는 당일 CRM 등록, 상담 후 주요 내용 즉시 기록, 계약 실패도 삭제하지 말고 이유 기록
-· 매일 확인: 신규/미답변 문의·정보 대기 고객·작성/미발송 견적·재연락 예정·계약 대기·일정 조율·대표 결정 필요
-· 학생 신분으로 가용시간이 변동될 수 있으므로 중요도 높은 업무(상지대 지원 마감·패키지·CRM)부터 하고, 초과분은 다음 주로 이월
+          <t>· 상품·상담·견적·계약·사후관리가 모두 하나의 CRM 안에서 연결되도록 구성합니다
+· 모든 고객에게 반드시 3가지: ① 현재 진행상태 ② 담당자 ③ 다음 행동·예정일
+· 신규 문의는 당일 CRM 등록, 상담 후 즉시 기록, 계약 실패도 삭제하지 말고 이유 기록
+· 진행상황 점검·지연고객 관리는 사람이 매일 수기로 하지 않고 AI 자동화로 처리되도록 설계합니다
+· 학생 신분으로 가용시간이 변동될 수 있으므로 중요도 높은 업무(상지대 지원 마감·패키지·CRM)부터 하고 초과분은 다음 주로 이월
 · 세부 마감은 별도로 두지 않고 금요일 주간보고로 정리 (단, 상지대 지원은 공고 마감을 우선)</t>
         </is>
       </c>
@@ -2085,9 +2085,8 @@
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>① 대상 고객(건물주·임대인·관리자·공인중개사·입주/퇴실 예정 고객)과 적용 대상(상가·사무실·원룸/오피스텔·소형건물)을 정의합니다.
-② 기본 서비스 범위·추가 옵션·제외 항목, 입실/퇴실 패키지 차이, 진행 순서·소요시간·가능 지역·고객 준비사항·완료 결과물·문제 처리 기준을 정리합니다.
-③ 산출물을 만듭니다: 내부용 상품정의서 / 고객용 1페이지 소개서 / 상담용 설명문 / 진행순서 안내 / FAQ / 기본가격·추가옵션표 / 고객 필수정보 목록.</t>
+          <t>① 대상 고객·적용 대상, 기본 서비스 범위·추가 옵션·제외 항목, 입실/퇴실 차이, 진행 순서·소요시간·가능 지역·고객 준비사항·완료 결과물·문제 처리 기준을 정리합니다.
+② 산출물을 만듭니다: 내부용 상품정의서 / 고객용 1페이지 소개서 / 상담용 설명문 / 진행순서 안내 / FAQ / 기본가격·추가옵션표 / 고객 필수정보 목록.</t>
         </is>
       </c>
       <c r="F28" s="47" t="inlineStr">
@@ -2111,10 +2110,10 @@
         </is>
       </c>
       <c r="J28" s="114" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.18</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="29" ht="123" customHeight="1" s="49">
@@ -2123,24 +2122,25 @@
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>CRM 구축 및 관리</t>
+          <t>CRM 구축·관리 (운영 프로세스 상품화 반영)</t>
         </is>
       </c>
       <c r="D29" s="47" t="inlineStr">
         <is>
-          <t>정리한 업무 흐름을 CRM에 실제로 적용해 고객을 단계별로 관리합니다.</t>
+          <t>정리해 둔 운영 프로세스를 상품화 형태(상품정의서·소개서·상담문구·가격표처럼)로 더 세분화해 CRM에 반영하고, 상품·상담·견적·계약·사후관리가 모두 CRM 안에서 이뤄지도록 구성합니다.</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>① CRM 진행 14단계(잠재→신규문의→상담→현장정보→견적준비→견적발송→검토→계약확정→일정조율→서비스진행→완료확인→결제완료→리뷰요청→사후관리)를 반영합니다.
-② 고객별 필수 입력정보(고객명·연락처·유형·건물/주소/용도·면적·층수·입퇴실 예정일·필요 서비스·채널·상담내용·견적/계약금액·진행상태·담당자·다음연락일·서류/사진 링크·특이사항·계약여부·실패이유)를 정의합니다.
-③ 관리 기준을 적용합니다: 신규 당일 등록·담당자 지정·다음 연락일 입력·상담 즉시 기록·계약 실패도 이유 기록·개인정보는 공개 링크 금지.</t>
+          <t>① CRM 진행 14단계와 고객별 필수 입력정보(고객·연락처·유형·건물/주소/용도·면적·입퇴실일·필요서비스·채널·상담내용·견적/계약금액·진행상태·담당자·다음연락일·서류/사진 링크·특이사항·계약여부·실패이유)를 반영합니다.
+② 운영 프로세스를 서비스·단계별로 세분화해 CRM 항목·화면 구성으로 만듭니다.
+③ 상품·상담·견적·계약·사후관리가 하나의 CRM 안에서 연결되도록 구조화합니다.
+④ 관리기준(당일 등록·담당자 지정·다음 연락일·실패 이유 기록·개인정보 공개 금지)을 적용합니다.</t>
         </is>
       </c>
       <c r="F29" s="47" t="inlineStr">
         <is>
-          <t>02_김현진_CRM_구축관리_W31_v1.xlsx</t>
+          <t>02_김현진_CRM_구축_프로세스반영_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -2162,7 +2162,7 @@
         <v>5</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="30" ht="84" customHeight="1" s="49">
@@ -2171,24 +2171,25 @@
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>고객 상담 프로세스·문구 정비</t>
+          <t>고객센터용 상담 대응 페이지 구축</t>
         </is>
       </c>
       <c r="D30" s="47" t="inlineStr">
         <is>
-          <t>문의가 오면 고객 상황을 정확히 파악하고 필요한 정보를 CRM에 기록할 수 있도록 상담 체계를 만듭니다.</t>
+          <t>고객 상담이 왔을 때 어떻게 대처하는지를 미리 정의해 고객센터용으로 별도 구축합니다. (CRM·마케팅과 구분되는 고객센터 축)</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>① 상담 시 확인할 내용(입실/퇴실·위치·유형·면적·희망일·현장상태·청소범위·폐기물·추가서비스·주차/출입·엘리베이터·사진 제공·예산/완료기준)을 체크리스트로 정리합니다.
-② 상담 후 처리(상담 기록·요청사항 요약·추가 사진/서류 요청·현장방문 판단·견적 담당/일정 지정·다음 과정 안내·다음 연락일 등록)를 정합니다.
-③ 상담 문구 세트(첫 문의 답변·부재 시 문자·사진 요청·추가정보 요청·현장방문 제안·견적 발송/확인·보류 재연락·계약 확정·일정 안내·완료 후 리뷰 요청)를 작성합니다.</t>
+          <t>① 문의 유형별 대응 시나리오(첫 응대·부재 시 문자·정보/사진 요청·현장방문 제안·견적/계약 안내·불만·환불/재작업 요청)를 정리합니다.
+② 상담 확인 체크리스트(입퇴실·위치·유형·면적·희망일·현장상태·청소범위·폐기물·주차/출입·예산/완료기준)를 만듭니다.
+③ 상담 문구 세트(첫 문의·부재 문자·사진 요청·추가정보 요청·현장방문·견적 발송/확인·보류 재연락·계약 확정·일정 안내·리뷰 요청)를 작성합니다.
+④ 누구나 같은 기준으로 응대할 수 있도록 고객센터용 페이지/문서로 정리합니다.</t>
         </is>
       </c>
       <c r="F30" s="47" t="inlineStr">
         <is>
-          <t>03_김현진_상담_프로세스_문구_W31_v1.xlsx</t>
+          <t>03_김현진_고객센터_상담대응_구축_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2207,7 +2208,7 @@
         </is>
       </c>
       <c r="J30" s="114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K30" s="19" t="n">
         <v>0.12</v>
@@ -2219,19 +2220,19 @@
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
-          <t>견적 및 계약 진행 정비</t>
+          <t>견적·계약 진행 정비 (CRM 내)</t>
         </is>
       </c>
       <c r="D31" s="47" t="inlineStr">
         <is>
-          <t>견적 작성·발송·계약 확정 절차를 정비합니다.</t>
+          <t>견적 작성·발송·계약 확정 절차를 CRM 흐름 안에서 정비합니다.</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
           <t>① 견적 전 확인사항(서비스 범위·면적·오염상태·난이도·인원·작업시간·외주/협력비·소모품·이동·폐기물·옵션·예상 원가/마진)을 정리합니다.
-② 견적 발송 후 관리(CRM 견적금액·견적서 링크·발송일·유효기간·고객 확인·익일 확인·3일 후 재연락·할인요청 기록·가격변경은 대표 승인·실패 이유 기록)를 정합니다.
-③ 계약 확정 후 절차(계약금액 확정·범위 재확인·일정·결제방식·고객 준비사항 안내·문서 CRM 연결·담당자 전달·변경/취소 조건 안내)를 정리합니다.</t>
+② 견적 발송 후 관리(CRM 견적금액·견적서 링크·발송일·유효기간·고객 확인·익일 확인·3일 후 재연락·할인요청 기록·가격변경은 대표 승인·실패 이유 기록).
+③ 계약 확정 후 절차(계약금액·범위 재확인·일정·결제방식·고객 준비사항·문서 CRM 연결·담당자 전달·변경/취소 조건 안내).</t>
         </is>
       </c>
       <c r="F31" s="47" t="inlineStr">
@@ -2267,24 +2268,25 @@
       </c>
       <c r="C32" s="47" t="inlineStr">
         <is>
-          <t>잠재고객·제휴처 영업</t>
+          <t>문의~계약 진행상황 관리 AI 자동화</t>
         </is>
       </c>
       <c r="D32" s="47" t="inlineStr">
         <is>
-          <t>우선 영업 대상과 제휴처를 등록하고 영업을 시작합니다. 제휴 조건·소개 수수료는 대표 보고 후 결정합니다.</t>
+          <t>진행상황 점검·지연고객 관리를 사람이 매일 수기로 하지 않고 AI 자동화로 처리되도록 설계·구축합니다.</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>① 우선 대상(건물주·임대인·관리업체·공인중개사·오피스텔 관리자·이사/청소/인테리어/폐기물 업체·이전 예정 사업자)을 등록합니다.
-② 대상별 기록(업체/고객명·지역·담당자·연락처·업종·예상 서비스·제휴 가능성·첫 연락일·상담내용·반응·자료 발송·다음 연락일·제휴 조건·실적)을 관리합니다.
-③ 제휴 제안 내용(고객 연결·공동 안내·상호 소개·서비스별 협력·소개비/제휴 방식·장기 협력)을 준비하되, 조건·수수료는 대표 보고 후 확정합니다.</t>
+          <t>① 자동 점검 대상을 정의합니다(신규/미답변 문의·정보 대기·미발송 견적·재연락 예정·계약 대기·일정 조율·지연 고객).
+② 자동화 규칙·트리거·알림 방식을 정의합니다(예: 다음 연락일 도래·N일 무응답 시 알림, 대표 결정 필요 건 자동 표시).
+③ 기존 FM 자동화·CRM과 연동할 지점을 정의합니다.
+④ 1차로 동작하는 자동화 또는 바로 실행 가능한 자동화 설계안을 제출합니다.</t>
         </is>
       </c>
       <c r="F32" s="47" t="inlineStr">
         <is>
-          <t>05_김현진_잠재고객_제휴영업_W31_v1.xlsx</t>
+          <t>05_김현진_진행상황_AI자동화_W31_v1.pdf</t>
         </is>
       </c>
       <c r="G32" s="108" t="inlineStr">
@@ -2303,34 +2305,35 @@
         </is>
       </c>
       <c r="J32" s="114" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="33" ht="90" customHeight="1" s="49">
       <c r="B33" s="17" t="n"/>
       <c r="C33" s="47" t="inlineStr">
         <is>
-          <t>문의~계약 전체 진행상황 관리</t>
+          <t>CRM 월간보고서 자동 산출 기능</t>
         </is>
       </c>
       <c r="D33" s="47" t="inlineStr">
         <is>
-          <t>문의 응대에 그치지 않고 각 고객이 현재 어디까지 진행됐는지 계속 관리합니다.</t>
+          <t>CRM에 쌓인 데이터를 매달 월간보고서 형식으로 받아볼 수 있게 만듭니다.</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>① 매일 점검(신규/미답변 문의·정보 대기·작성/미발송 견적·재연락 예정·계약 대기·일정 조율·대표 결정 필요)을 수행합니다.
-② 모든 고객에 3요소(진행상태·담당자·다음 행동/예정일)를 유지합니다.
-③ 지연 고객(무응답·자료 미제공·견적 후 무응답·계약 보류·일정 미확정)에 재연락 날짜를 정하고 결과를 CRM에 기록합니다.</t>
+          <t>① 월간보고서 항목을 정의합니다(신규문의·상담·견적·계약 수·계약금액·전환율·채널별 성과·계약 실패 이유·사후관리·다음 달 파이프라인).
+② CRM에서 월 단위로 자동 집계되는 구조를 설계합니다.
+③ 보고서 양식(요약+표) 1개를 확정합니다.
+④ 이번 달(또는 샘플) 1개월치 월간보고서 초안을 산출합니다.</t>
         </is>
       </c>
       <c r="F33" s="47" t="inlineStr">
         <is>
-          <t>06_김현진_진행상황_관리_W31_v1.xlsx</t>
+          <t>06_김현진_CRM_월간보고서_기능_W31_v1.xlsx</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2349,17 +2352,17 @@
         </is>
       </c>
       <c r="J33" s="114" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="34" ht="90" customHeight="1" s="49">
       <c r="B34" s="17" t="n"/>
       <c r="C34" s="47" t="inlineStr">
         <is>
-          <t>입·퇴실 패키지 전체 과정 테스트</t>
+          <t>입·퇴실 패키지 전체 과정 테스트 (가상고객 1건)</t>
         </is>
       </c>
       <c r="D34" s="47" t="inlineStr">
@@ -2371,7 +2374,7 @@
         <is>
           <t>① 신규 문의→기본정보→상담→현장정보/사진→견적 작성/발송→계약 확정→일정→서비스 진행→완료 자료→결제 완료→리뷰 요청→사후관리까지 1건을 끝까지 진행합니다.
 ② 테스트 중 확인(빠진 정보·중복 항목·불명확한 단계·없는 서류/안내문·담당자 미지정·설명 어려운 내용·대표 승인 필요 지점)을 정리합니다.
-③ 결과를 CRM·업무 흐름에 반영합니다.</t>
+③ 결과를 CRM·업무 흐름·고객센터 대응에 반영합니다.</t>
         </is>
       </c>
       <c r="F34" s="47" t="inlineStr">
@@ -2398,7 +2401,7 @@
         <v>3</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="35" ht="90" customHeight="1" s="49">
@@ -2416,7 +2419,7 @@
       <c r="E35" s="1" t="inlineStr">
         <is>
           <t>① 먼저 확인: 지원사업명·지원금액·대상·신청 마감일·제출방법·가능 광고채널·자부담·집행기간·선결제/부가세·정산방식.
-② 신청서 초안 작성(회사/대표/사업자 정보·신청 목적·서비스 및 입퇴실 패키지 소개·광고 필요성·목표 고객·채널·100만 원 사용계획·기간·기대효과·예상 문의/계약 수·성과관리 방법).
+② 신청서 초안 작성(회사/대표/사업자 정보·신청 목적·서비스 및 입퇴실 패키지 소개·광고 필요성·목표 고객·채널·100만 원 사용계획·기간·기대효과·예상 문의/계약·성과관리).
 ③ 첨부서류 확보(사업자등록증·통장사본·회사소개서·광고 견적서·집행계획서·개인정보 동의서·신청서 등)와 제출 전 검수(누락·회사/대표/사업자번호·예산 합계·기간·서명·파일명·형식·마감).
 ④ 최종본을 대표에게 먼저 확인받은 뒤 제출하고, 접수증/제출 완료 화면을 보관합니다.</t>
         </is>
@@ -2442,10 +2445,10 @@
         </is>
       </c>
       <c r="J35" s="114" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="36" ht="69" customHeight="1" s="49">

</xml_diff>